<commit_message>
1. 增加list node 查询node功能 2. 修改与agent的内部接口 3. 增加list business接口
git-svn-id: http://192.168.20.11/sequoiadb/trunk@14907 6121f079-4a18-41d3-8c30-8870a322f2c2
</commit_message>
<xml_diff>
--- a/internal_doc/03.开发设计/OM_web接口.xlsx
+++ b/internal_doc/03.开发设计/OM_web接口.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="6510" activeTab="5"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="6510" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="需求" sheetId="1" r:id="rId1"/>
@@ -281,7 +281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="313">
   <si>
     <t>需求</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -811,10 +811,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>rc=ok, 已经存在</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>INT32 catMainController::_ensureMetadata()</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -874,18 +870,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>remove_business_res</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>NA</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{rc, ???}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>返回跳转页面命令</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -894,10 +882,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>rest参数(响应最外层统一加上rc)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>网页跳转响应(GETFILE)(废除)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -923,10 +907,6 @@
   </si>
   <si>
     <t>通过接口获取（pAdptor-&gt;recvRequestBody( this, httpCommon, &amp;pFilePath, bodySize )）</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{rc,detail}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -972,11 +952,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>成功时：{rc}
-校验失败时：{rc,local} local为跳转文件login.html</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>获取cluster信息</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1005,19 +980,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{ClusterName, rc}</t>
-  </si>
-  <si>
-    <t>{ClusterName, rc}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>business_name=xxx&amp;ClusterName=xxx</t>
-  </si>
-  <si>
-    <t>{business_name, ClusterName, rc}</t>
-  </si>
-  <si>
     <t>replname</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1063,10 +1025,6 @@
   </si>
   <si>
     <t>host_info={ClusterName:cls1, host_info:[{IP, HostName, User, Passwd, SshPort:xxx, AgentPort:xxx},...], User:usr1, Passwd:Passwd1, SshPort:xxx, AgentPort:xxx}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{[{IP, HostName, rc, Firework, [Disk],[CPU]…}, ...]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1075,14 +1033,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[{IP, HostName, Ping:true, Ssh:false, HostName:"rhelt10", rc}, ...]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>rc=ok</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>"Config": [ { "HostName": "host1", "username": "sdbadmin", "userpasswd": "sdbadmin", "usergroup": "sdbadmin_group", "datagroupname": "", "dbpath": "/home/db2//standalone/11830", "svcname": "11830", ...} ],"BusinessName": "b1", "BusinessType": "sequoiadb", "ClusterType": "standalone","ClusterName": "c1","Property": [ { "Name": "username", "Type": "string", "Default": "sdbadmin", "Valid": "", "Display": "edit box", "Edit": "true", "Desc": "", "Level": "0", "WebName": "user_name",... }]</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1091,14 +1041,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ClusterName=cls1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ "rc": 0 }{ "BusinessList": [ { "BusinessType": "sequoiadb", "BusinessDesc": "haha" }, { "BusinessType": "sequoiasql", "BusinessDesc": "haha" } ] }</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>{BusinessType, BusinessName,ClusterType, ClusterName, "Config":[{"HostName":"host1","datagroupname":"", "dbpath":"/home/db2//standalone/11830", "svcname":"11830", ...}, ...] }]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1171,10 +1113,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>http://192.168.20.197:11814/?cmd=query host&amp;ClusterName=c1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>http://192.168.20.197:11814/?cmd=query business list</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1191,10 +1129,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{rc,local}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>query progress</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1211,19 +1145,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{ "rc": 0 }{ "ClusterName": "c1", "Desc": "" }</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>查询进度</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>查询进度响应</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ClusterName, rc, [IP, HostName, Firework, [Disk],[CPU]...]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1297,20 +1223,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>{"rc":0, "Detail":"","TaskID":"asd", "isFinish":true,"Status":"install/rollback","Progress":[{"Name":"Coord","TotalCount":7 "InstalledCount":100, "Desc":""}, {"Name":"Group1","TotalCount":3,"InstalledCount":50,"Desc":""},
-{"Name":"Group2","TotalCount":4,"InstalledCount":50,"Desc":""} ...]}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>http://192.168.20.197:11814/?cmd=scan host&amp;HostInfo={"ClusterName":"c1","HostInfo":[{"IP":"192.168.20.196","User":"root","Passwd":"sequoiad",SshPort:"22",AgentPort:"11790"}],"User":"root","Passwd":"sequoiadb",SshPort:"22",AgentPort:"11810"}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>http://192.168.20.197:11814/?cmd=query business template&amp;BusinessType=sequoiadb</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>{ "rc": 0 }{ "DeployMod": "standalone", "WebName": "standalone", "BusinessType": "sequoiadb", "Property": [ { "Name": "replicanum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "replica_num" }, { "Name": "datagroupnum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "data_group_num" }, { "Name": "catalognum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "1", "Level": "0", "WebName": "catalog_num" }, { "Name": "coordnum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "coord_num" }, { "Name": "transactionon", "Type": "string", "Default": "false", "Valid": "true,false", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "transactionon" } ] }{ "DeployMod": "distribution", "WebName": "distribution", "BusinessType": "sequoiadb", "Property": [ { "Name": "replicanum", "Type": "int", "Default": "3", "Valid": "1-7", "Display": "edit box", "Edit": "true", "Desc": "", "Level": "0", "WebName": "replica_num" }, { "Name": "datagroupnum", "Type": "int", "Default": "1", "Valid": "", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "data_group_num" }, { "Name": "catalognum", "Type": "int", "Default": "1", "Valid": "", "Display": "edit box", "Edit": "false", "Desc": "1", "Level": "0", "WebName": "catalog_num" }, { "Name": "coordnum", "Type": "int", "Default": "0", "Valid": "0-7", "Display": "edit box", "Edit": "false", "Desc": "0 means one coord each host", "Level": "0", "WebName": "coord_num" }, { "Name": "transactionon", "Type": "string", "Default": "false", "Valid": "true,false", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "transactionon" } ] }</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1543,6 +1460,135 @@
   </si>
   <si>
     <t>{"HostName":"", "IP":"", "User":"", "Passwd":"", "InstallPath":""}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>HostName=host1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://192.168.20.197:11814/?cmd=query host&amp;HostName=host1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获取host列表</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>list host</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获取host列表响应</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ "Rc": 0 }{ "HostName": "rhelt10" }</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> http://192.168.20.197:11814/?cmd=list host&amp;ClusterName=c1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ClusterName=c1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ClusterName=c1(or BusinessName=b1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ "Rc": 0 }{ "_id": { "$oid": "54096ec6f1ee34d0b015a6ce" }, "HostName": "rhelt10", "ClusterName": "c1", "IP": "192.168.20.197", "User": "root", "Password": "sequoiadb", "OS": { "Distributor": "Ubuntu", "Release": "12.04", "Bit": 64 }, "OM": { "Status": 0, "Version": "" }, "Memory": { "Model": "", "Size": 2003, "Free": 916, "Unit": "M" }, "Disk": [ { "Name": "/dev/mapper/vgdata-lvdata1", "Mount": "/home/mount/", "Size": 32529, "Free": 6525, "Unit": "M", "Used": 1 } ], "CPU": [ { "ID": "", "Model": "", "Core": 1, "Freq": "2.00GHz" } ], "Net": [ { "Name": "lo", "Model": "", "Bandwidth": "", "IP": "127.0.0.1" }, { "Name": "eth0", "Model": "", "Bandwidth": "", "IP": "192.168.20.197" } ], "Service": [ { "Name": "", "Status": 0, "Version": "" } ], "Safety": { "Name": "", "Context": "", "Status": 0 }, "InstallPath": "/opt/sequoiadb/", "AgentPort": "11790" }</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>查询business列表</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>查询business列表响应</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>list business</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>192.168.20.197:11814/?cmd=list business&amp;ClusterName=c1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{ "Rc": 0 }{ "BusinessName": "b1" },{}...</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BusinessName=xxx</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{Rc}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://192.168.20.197:11814/?cmd=remove business&amp;BusinessName=b1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>删除集群响应</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rc=ok, 已经存在</t>
+  </si>
+  <si>
+    <t>{ "Rc": 0 }{ "ClusterName": "c1", "Desc": "" }</t>
+  </si>
+  <si>
+    <t>[{IP, HostName, Ping:true, Ssh:false, HostName:"rhelt10", Rc}, ...]</t>
+  </si>
+  <si>
+    <t>Rc=ok</t>
+  </si>
+  <si>
+    <t>{[{IP, HostName, Rc, Firework, [Disk],[CPU]…}, ...]}</t>
+  </si>
+  <si>
+    <t>{ "Rc": 0 }{ "BusinessList": [ { "BusinessType": "sequoiadb", "BusinessDesc": "haha" }, { "BusinessType": "sequoiasql", "BusinessDesc": "haha" } ] }</t>
+  </si>
+  <si>
+    <t>{ "Rc": 0 }{ "DeployMod": "standalone", "WebName": "standalone", "BusinessType": "sequoiadb", "Property": [ { "Name": "replicanum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "replica_num" }, { "Name": "datagroupnum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "data_group_num" }, { "Name": "catalognum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "1", "Level": "0", "WebName": "catalog_num" }, { "Name": "coordnum", "Type": "int", "Default": "1", "Valid": "1", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "coord_num" }, { "Name": "transactionon", "Type": "string", "Default": "false", "Valid": "true,false", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "transactionon" } ] }{ "DeployMod": "distribution", "WebName": "distribution", "BusinessType": "sequoiadb", "Property": [ { "Name": "replicanum", "Type": "int", "Default": "3", "Valid": "1-7", "Display": "edit box", "Edit": "true", "Desc": "", "Level": "0", "WebName": "replica_num" }, { "Name": "datagroupnum", "Type": "int", "Default": "1", "Valid": "", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "data_group_num" }, { "Name": "catalognum", "Type": "int", "Default": "1", "Valid": "", "Display": "edit box", "Edit": "false", "Desc": "1", "Level": "0", "WebName": "catalog_num" }, { "Name": "coordnum", "Type": "int", "Default": "0", "Valid": "0-7", "Display": "edit box", "Edit": "false", "Desc": "0 means one coord each host", "Level": "0", "WebName": "coord_num" }, { "Name": "transactionon", "Type": "string", "Default": "false", "Valid": "true,false", "Display": "edit box", "Edit": "false", "Desc": "", "Level": "0", "WebName": "transactionon" } ] }</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{Rc, ???}</t>
+  </si>
+  <si>
+    <t>{"Rc":0, "Detail":"","TaskID":"asd", "isFinish":true,"Status":"install/rollback","Progress":[{"Name":"Coord","TotalCount":7 "InstalledCount":100, "Desc":""}, {"Name":"Group1","TotalCount":3,"InstalledCount":50,"Desc":""},
+{"Name":"Group2","TotalCount":4,"InstalledCount":50,"Desc":""} ...]}</t>
+  </si>
+  <si>
+    <t>成功时：{Rc}
+校验失败时：{Rc,local} local为跳转文件login.html</t>
+  </si>
+  <si>
+    <t>{Rc,local}</t>
+  </si>
+  <si>
+    <t>{Rc,detail}</t>
+  </si>
+  <si>
+    <t>{ClusterName, Rc}</t>
+  </si>
+  <si>
+    <t>rest参数(响应最外层统一加上Rc)</t>
+  </si>
+  <si>
+    <t>删除host</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>remove host</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1791,7 +1837,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1847,10 +1893,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1877,6 +1919,10 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1895,14 +1941,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3106,7 +3159,7 @@
     <row r="14" spans="1:12">
       <c r="A14" s="14"/>
       <c r="B14" s="14" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="C14" s="14">
         <v>11811</v>
@@ -3128,7 +3181,7 @@
     <row r="15" spans="1:12">
       <c r="A15" s="14"/>
       <c r="B15" s="14" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="C15" s="14">
         <v>11812</v>
@@ -3150,7 +3203,7 @@
     <row r="16" spans="1:12">
       <c r="A16" s="14"/>
       <c r="B16" s="14" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C16" s="14">
         <v>11813</v>
@@ -3172,7 +3225,7 @@
     <row r="17" spans="1:12">
       <c r="A17" s="14"/>
       <c r="B17" s="14" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="C17" s="14">
         <v>11814</v>
@@ -3194,7 +3247,7 @@
     <row r="18" spans="1:12">
       <c r="A18" s="14"/>
       <c r="B18" s="14" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="C18" s="14">
         <v>3</v>
@@ -3218,7 +3271,7 @@
     <row r="19" spans="1:12">
       <c r="A19" s="14"/>
       <c r="B19" s="14" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>95</v>
@@ -3242,7 +3295,7 @@
     <row r="20" spans="1:12">
       <c r="A20" s="14"/>
       <c r="B20" s="14" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="C20" s="14">
         <v>64</v>
@@ -3255,7 +3308,7 @@
         <v>102</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="H20" s="14"/>
       <c r="I20" s="14"/>
@@ -3266,7 +3319,7 @@
     <row r="21" spans="1:12">
       <c r="A21" s="14"/>
       <c r="B21" s="14" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="C21" s="14">
         <v>20</v>
@@ -3279,7 +3332,7 @@
         <v>102</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="H21" s="14"/>
       <c r="I21" s="14"/>
@@ -3290,7 +3343,7 @@
     <row r="22" spans="1:12">
       <c r="A22" s="14"/>
       <c r="B22" s="14" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>109</v>
@@ -3338,7 +3391,7 @@
     <row r="24" spans="1:12">
       <c r="A24" s="14"/>
       <c r="B24" s="16" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="C24" s="11">
         <v>1</v>
@@ -3360,7 +3413,7 @@
     <row r="25" spans="1:12" s="19" customFormat="1">
       <c r="A25" s="16"/>
       <c r="B25" s="16" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="C25" s="11">
         <v>10000</v>
@@ -3667,10 +3720,10 @@
   <dimension ref="A1:F74"/>
   <sheetFormatPr defaultRowHeight="12"/>
   <cols>
-    <col min="1" max="1" width="26" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.75" style="3" customWidth="1"/>
-    <col min="3" max="3" width="45.125" style="10" customWidth="1"/>
-    <col min="4" max="4" width="52.25" style="10" customWidth="1"/>
+    <col min="1" max="1" width="22.375" style="10" customWidth="1"/>
+    <col min="2" max="2" width="22.625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="54.125" style="10" customWidth="1"/>
+    <col min="4" max="4" width="57.375" style="10" customWidth="1"/>
     <col min="5" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
@@ -3689,10 +3742,10 @@
         <v>119</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>151</v>
+        <v>310</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>1</v>
@@ -3702,16 +3755,16 @@
     </row>
     <row r="3" spans="1:6" ht="48">
       <c r="A3" s="9" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>227</v>
+        <v>210</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -3722,10 +3775,10 @@
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>179</v>
+        <v>309</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>130</v>
+        <v>297</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
@@ -3740,30 +3793,30 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="9" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>228</v>
+        <v>211</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="9" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="9" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>230</v>
+        <v>298</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
@@ -3776,72 +3829,68 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" spans="1:6" ht="60">
-      <c r="A9" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="C9" s="9" t="s">
+    <row r="9" spans="1:6" s="45" customFormat="1">
+      <c r="A9" s="43" t="s">
+        <v>236</v>
+      </c>
+      <c r="B9" s="44" t="s">
         <v>239</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="1:6" ht="24">
-      <c r="A10" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="9"/>
-      <c r="B11" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
+      <c r="C9" s="43" t="s">
+        <v>234</v>
+      </c>
+      <c r="D9" s="43" t="s">
+        <v>240</v>
+      </c>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+    </row>
+    <row r="10" spans="1:6" s="45" customFormat="1">
+      <c r="A10" s="43" t="s">
+        <v>296</v>
+      </c>
+      <c r="B10" s="44"/>
+      <c r="C10" s="43" t="s">
+        <v>294</v>
+      </c>
+      <c r="D10" s="43"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+    </row>
+    <row r="11" spans="1:6" s="49" customFormat="1">
+      <c r="A11" s="47"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="47"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
     </row>
     <row r="12" spans="1:6" ht="60">
       <c r="A12" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>193</v>
+        <v>220</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>263</v>
+        <v>221</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
     </row>
-    <row r="13" spans="1:6" ht="102.75" customHeight="1">
+    <row r="13" spans="1:6" ht="24">
       <c r="A13" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="9" t="s">
-        <v>194</v>
+        <v>299</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>262</v>
+        <v>300</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
@@ -3849,74 +3898,76 @@
     <row r="14" spans="1:6">
       <c r="A14" s="9"/>
       <c r="B14" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
     </row>
-    <row r="15" spans="1:6" ht="120" customHeight="1">
+    <row r="15" spans="1:6" ht="60">
       <c r="A15" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>253</v>
+        <v>183</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" ht="228">
       <c r="A16" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="D16" s="9"/>
+        <v>301</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>241</v>
+      </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="9"/>
       <c r="B17" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
     </row>
-    <row r="18" spans="1:6" ht="27">
+    <row r="18" spans="1:6" ht="204">
       <c r="A18" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>220</v>
+        <v>232</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>243</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="1:6" ht="24">
+    <row r="19" spans="1:6">
       <c r="A19" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="9" t="s">
-        <v>233</v>
+        <v>309</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="4"/>
@@ -3925,7 +3976,7 @@
     <row r="20" spans="1:6">
       <c r="A20" s="9"/>
       <c r="B20" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
@@ -3934,155 +3985,139 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="9" t="s">
-        <v>135</v>
+        <v>280</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="C21" s="9"/>
+        <v>281</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>286</v>
+      </c>
       <c r="D21" s="9" t="s">
-        <v>221</v>
+        <v>284</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
-    <row r="22" spans="1:6" ht="36">
+    <row r="22" spans="1:6">
       <c r="A22" s="9" t="s">
-        <v>136</v>
+        <v>282</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>201</v>
-      </c>
+        <v>283</v>
+      </c>
+      <c r="D22" s="9"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="9"/>
-      <c r="B23" s="4" t="s">
-        <v>133</v>
-      </c>
+      <c r="B23" s="4"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" spans="1:6" ht="24">
+    <row r="24" spans="1:6">
       <c r="A24" s="9" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>234</v>
+        <v>195</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>235</v>
+        <v>278</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>242</v>
+        <v>279</v>
       </c>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" spans="1:6" ht="240">
+    <row r="25" spans="1:6" ht="180">
       <c r="A25" s="9" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>243</v>
-      </c>
+        <v>287</v>
+      </c>
+      <c r="D25" s="9"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="9"/>
-      <c r="B26" s="4" t="s">
-        <v>133</v>
-      </c>
+      <c r="B26" s="4"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="1:6" ht="84">
+    <row r="27" spans="1:6">
       <c r="A27" s="9" t="s">
-        <v>139</v>
+        <v>311</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>244</v>
-      </c>
+        <v>312</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="1:6" ht="120">
-      <c r="A28" s="9" t="s">
-        <v>140</v>
-      </c>
+    <row r="28" spans="1:6">
+      <c r="A28" s="9"/>
       <c r="B28" s="4"/>
-      <c r="C28" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>198</v>
-      </c>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="9"/>
       <c r="B29" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:6" ht="144">
+    <row r="30" spans="1:6">
       <c r="A30" s="9" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>202</v>
-      </c>
+        <v>224</v>
+      </c>
+      <c r="C30" s="9"/>
       <c r="D30" s="9" t="s">
-        <v>270</v>
+        <v>205</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" ht="36">
       <c r="A31" s="9" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="9" t="s">
-        <v>148</v>
+        <v>206</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>120</v>
+        <v>302</v>
       </c>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="9"/>
-      <c r="B32" s="4"/>
+      <c r="B32" s="4" t="s">
+        <v>132</v>
+      </c>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
       <c r="E32" s="4"/>
@@ -4090,95 +4125,111 @@
     </row>
     <row r="33" spans="1:6" ht="24">
       <c r="A33" s="9" t="s">
-        <v>231</v>
+        <v>136</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
     </row>
-    <row r="34" spans="1:6" ht="96">
+    <row r="34" spans="1:6" ht="228">
       <c r="A34" s="9" t="s">
-        <v>232</v>
+        <v>137</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="D34" s="9"/>
+        <v>184</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>303</v>
+      </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="9"/>
-      <c r="B35" s="4"/>
+      <c r="B35" s="4" t="s">
+        <v>132</v>
+      </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
-    <row r="36" spans="1:6" ht="24">
+    <row r="36" spans="1:6" ht="84">
       <c r="A36" s="9" t="s">
-        <v>258</v>
+        <v>138</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>254</v>
+        <v>196</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>255</v>
+        <v>217</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>256</v>
+        <v>223</v>
       </c>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" ht="108">
       <c r="A37" s="9" t="s">
-        <v>259</v>
+        <v>139</v>
       </c>
       <c r="B37" s="4"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
+      <c r="C37" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>185</v>
+      </c>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="9"/>
-      <c r="B38" s="4"/>
+      <c r="B38" s="4" t="s">
+        <v>132</v>
+      </c>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="1:6" ht="24">
+    <row r="39" spans="1:6" ht="132">
       <c r="A39" s="9" t="s">
-        <v>257</v>
+        <v>140</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>260</v>
+        <v>197</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>255</v>
+        <v>187</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="9"/>
+      <c r="A40" s="9" t="s">
+        <v>141</v>
+      </c>
       <c r="B40" s="4"/>
-      <c r="C40" s="9"/>
-      <c r="D40" s="9"/>
+      <c r="C40" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
     </row>
@@ -4191,85 +4242,138 @@
       <c r="F41" s="4"/>
     </row>
     <row r="42" spans="1:6">
-      <c r="A42" s="9"/>
+      <c r="A42" s="9" t="s">
+        <v>288</v>
+      </c>
       <c r="B42" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C42" s="9"/>
-      <c r="D42" s="9"/>
+        <v>290</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>291</v>
+      </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>145</v>
-      </c>
+        <v>289</v>
+      </c>
+      <c r="B43" s="4"/>
       <c r="C43" s="9" t="s">
-        <v>180</v>
+        <v>292</v>
       </c>
       <c r="D43" s="9"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
     </row>
     <row r="44" spans="1:6">
-      <c r="A44" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>181</v>
-      </c>
+      <c r="A44" s="9"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="9"/>
       <c r="D44" s="9"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="43"/>
-      <c r="B45" s="44"/>
-      <c r="C45" s="43"/>
-      <c r="D45" s="43"/>
-      <c r="E45" s="44"/>
-      <c r="F45" s="44"/>
-    </row>
-    <row r="46" spans="1:6" s="4" customFormat="1">
-      <c r="A46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-    </row>
-    <row r="47" spans="1:6" s="4" customFormat="1">
-      <c r="A47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="9"/>
-    </row>
-    <row r="48" spans="1:6" s="4" customFormat="1">
-      <c r="A48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="9"/>
-    </row>
-    <row r="49" spans="1:6" s="4" customFormat="1">
-      <c r="A49" s="9"/>
-      <c r="C49" s="9"/>
+    <row r="45" spans="1:6" s="46" customFormat="1">
+      <c r="A45" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+    </row>
+    <row r="46" spans="1:6" s="46" customFormat="1">
+      <c r="A46" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="B46" s="2"/>
+      <c r="C46" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="D46" s="5"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+    </row>
+    <row r="47" spans="1:6" s="49" customFormat="1">
+      <c r="A47" s="47"/>
+      <c r="B47" s="48"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="47"/>
+      <c r="E47" s="48"/>
+      <c r="F47" s="48"/>
+    </row>
+    <row r="48" spans="1:6" ht="24">
+      <c r="A48" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+    </row>
+    <row r="49" spans="1:6" ht="84">
+      <c r="A49" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B49" s="4"/>
+      <c r="C49" s="9" t="s">
+        <v>305</v>
+      </c>
       <c r="D49" s="9"/>
-    </row>
-    <row r="50" spans="1:6" s="4" customFormat="1">
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50" s="9"/>
+      <c r="B50" s="4"/>
       <c r="C50" s="9"/>
       <c r="D50" s="9"/>
-    </row>
-    <row r="51" spans="1:6" s="4" customFormat="1">
-      <c r="A51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="9"/>
-    </row>
-    <row r="52" spans="1:6" s="4" customFormat="1">
-      <c r="A52" s="9"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+    </row>
+    <row r="52" spans="1:6" ht="24">
+      <c r="A52" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="B52" s="4"/>
       <c r="C52" s="9"/>
       <c r="D52" s="9"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
     </row>
     <row r="53" spans="1:6" s="4" customFormat="1">
       <c r="A53" s="9"/>
@@ -4282,29 +4386,29 @@
       <c r="D54" s="9"/>
     </row>
     <row r="55" spans="1:6">
-      <c r="A55" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="B55" s="46" t="s">
-        <v>206</v>
-      </c>
-      <c r="C55" s="45" t="s">
-        <v>147</v>
-      </c>
-      <c r="D55" s="45"/>
-      <c r="E55" s="46"/>
-      <c r="F55" s="46"/>
+      <c r="A55" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="B55" s="36" t="s">
+        <v>191</v>
+      </c>
+      <c r="C55" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="D55" s="35"/>
+      <c r="E55" s="36"/>
+      <c r="F55" s="36"/>
     </row>
     <row r="56" spans="1:6" ht="24">
       <c r="A56" s="9" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="9" t="s">
-        <v>170</v>
+        <v>306</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
@@ -4319,54 +4423,54 @@
     </row>
     <row r="58" spans="1:6" ht="24">
       <c r="A58" s="9" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>237</v>
+        <v>218</v>
       </c>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="9" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="9" t="s">
-        <v>225</v>
+        <v>307</v>
       </c>
       <c r="D59" s="9"/>
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
     </row>
-    <row r="60" spans="1:6" ht="36">
+    <row r="60" spans="1:6" ht="24">
       <c r="A60" s="9" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="E60" s="4"/>
       <c r="F60" s="4"/>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" s="9" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>219</v>
+        <v>204</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
@@ -4381,95 +4485,95 @@
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
     </row>
-    <row r="63" spans="1:6">
-      <c r="A63" s="5" t="s">
+    <row r="63" spans="1:6" s="49" customFormat="1">
+      <c r="A63" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="B63" s="48"/>
+      <c r="C63" s="47" t="s">
+        <v>308</v>
+      </c>
+      <c r="D63" s="47"/>
+      <c r="E63" s="48"/>
+      <c r="F63" s="48"/>
+    </row>
+    <row r="64" spans="1:6" s="49" customFormat="1" ht="24">
+      <c r="A64" s="47" t="s">
+        <v>156</v>
+      </c>
+      <c r="B64" s="48"/>
+      <c r="C64" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="D64" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="E64" s="48"/>
+      <c r="F64" s="48"/>
+    </row>
+    <row r="65" spans="1:6" s="49" customFormat="1" ht="24">
+      <c r="A65" s="47" t="s">
+        <v>153</v>
+      </c>
+      <c r="B65" s="48" t="s">
+        <v>158</v>
+      </c>
+      <c r="C65" s="47" t="s">
+        <v>154</v>
+      </c>
+      <c r="D65" s="47"/>
+      <c r="E65" s="48"/>
+      <c r="F65" s="48"/>
+    </row>
+    <row r="66" spans="1:6" s="49" customFormat="1" ht="48">
+      <c r="A66" s="47" t="s">
+        <v>157</v>
+      </c>
+      <c r="B66" s="48" t="s">
+        <v>158</v>
+      </c>
+      <c r="C66" s="47" t="s">
+        <v>161</v>
+      </c>
+      <c r="D66" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="E66" s="48"/>
+      <c r="F66" s="48"/>
+    </row>
+    <row r="67" spans="1:6" s="49" customFormat="1" ht="36">
+      <c r="A67" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="B67" s="48" t="s">
+        <v>158</v>
+      </c>
+      <c r="C67" s="47" t="s">
         <v>160</v>
       </c>
-      <c r="B63" s="2"/>
-      <c r="C63" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="D63" s="5"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-    </row>
-    <row r="64" spans="1:6" ht="24">
-      <c r="A64" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="B64" s="2"/>
-      <c r="C64" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-    </row>
-    <row r="65" spans="1:6" ht="24">
-      <c r="A65" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="D65" s="5"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-    </row>
-    <row r="66" spans="1:6" ht="60">
-      <c r="A66" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C66" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="D66" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
-    </row>
-    <row r="67" spans="1:6" ht="48">
-      <c r="A67" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C67" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="D67" s="5"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-    </row>
-    <row r="68" spans="1:6" s="21" customFormat="1">
-      <c r="A68" s="25" t="s">
-        <v>152</v>
-      </c>
-      <c r="B68" s="26"/>
-      <c r="C68" s="25"/>
-      <c r="D68" s="25" t="s">
-        <v>150</v>
-      </c>
-      <c r="E68" s="26"/>
-      <c r="F68" s="26"/>
-    </row>
-    <row r="69" spans="1:6">
-      <c r="A69" s="5"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
+      <c r="D67" s="47"/>
+      <c r="E67" s="48"/>
+      <c r="F67" s="48"/>
+    </row>
+    <row r="68" spans="1:6" s="21" customFormat="1" ht="24">
+      <c r="A68" s="50" t="s">
+        <v>148</v>
+      </c>
+      <c r="B68" s="51"/>
+      <c r="C68" s="50"/>
+      <c r="D68" s="50" t="s">
+        <v>147</v>
+      </c>
+      <c r="E68" s="51"/>
+      <c r="F68" s="51"/>
+    </row>
+    <row r="69" spans="1:6" s="49" customFormat="1">
+      <c r="A69" s="47"/>
+      <c r="B69" s="48"/>
+      <c r="C69" s="47"/>
+      <c r="D69" s="47"/>
+      <c r="E69" s="48"/>
+      <c r="F69" s="48"/>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" s="9"/>
@@ -4530,18 +4634,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="40.5">
       <c r="B8" s="23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -4563,195 +4667,195 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>225</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>247</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="67.5">
+      <c r="A2" s="28" t="s">
+        <v>231</v>
+      </c>
+      <c r="B2" s="29" t="s">
+        <v>245</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>229</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="E2" s="30" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="29"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+    </row>
+    <row r="4" spans="1:5" ht="27">
+      <c r="A4" s="29" t="s">
+        <v>244</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>277</v>
+      </c>
+      <c r="D4" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="E4" s="30" t="s">
         <v>248</v>
       </c>
-      <c r="B1" s="27" t="s">
-        <v>246</v>
-      </c>
-      <c r="C1" s="28" t="s">
-        <v>247</v>
-      </c>
-      <c r="D1" s="28" t="s">
-        <v>268</v>
-      </c>
-      <c r="E1" s="28" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="67.5">
-      <c r="A2" s="30" t="s">
-        <v>252</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>266</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>250</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>249</v>
-      </c>
-      <c r="E2" s="32" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="31"/>
-      <c r="B3" s="31"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-    </row>
-    <row r="4" spans="1:5" ht="27">
-      <c r="A4" s="31" t="s">
-        <v>265</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="30" t="s">
-        <v>298</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>267</v>
-      </c>
-      <c r="E4" s="32" t="s">
-        <v>269</v>
-      </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="31"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="31"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="31"/>
-      <c r="B8" s="31"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
+      <c r="A8" s="29"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="31"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="31"/>
-      <c r="B10" s="31"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
+      <c r="A10" s="29"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="31"/>
-      <c r="B11" s="31"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="31"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="31"/>
-      <c r="B13" s="31"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
+      <c r="A13" s="29"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="31"/>
-      <c r="B14" s="31"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
+      <c r="A14" s="29"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="31"/>
-      <c r="B15" s="31"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="31"/>
-      <c r="B16" s="31"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
+      <c r="A16" s="29"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="31"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
+      <c r="A17" s="29"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="31"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
+      <c r="A18" s="29"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="31"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="31"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
+      <c r="A20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="31"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
+      <c r="A21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="28"/>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="31"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
+      <c r="A22" s="29"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="31"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
+      <c r="A23" s="29"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -4772,163 +4876,163 @@
   <sheetData>
     <row r="1" spans="1:4" ht="27">
       <c r="A1" s="23" t="s">
-        <v>273</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="27">
       <c r="A2" s="23" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="26" t="s">
+        <v>269</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>270</v>
+      </c>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="31" t="s">
+        <v>253</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="31" t="s">
+        <v>254</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="31" t="s">
+        <v>255</v>
+      </c>
+      <c r="B7" s="27" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="28" t="s">
-        <v>290</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>291</v>
-      </c>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="33" t="s">
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="31" t="s">
+        <v>256</v>
+      </c>
+      <c r="B8" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="31" t="s">
+        <v>257</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="31" t="s">
+        <v>258</v>
+      </c>
+      <c r="B10" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="31" t="s">
+        <v>259</v>
+      </c>
+      <c r="B11" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="31" t="s">
+        <v>260</v>
+      </c>
+      <c r="B12" s="27" t="s">
         <v>274</v>
       </c>
-      <c r="B5" s="29" t="s">
-        <v>289</v>
-      </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="33" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="31" t="s">
+        <v>265</v>
+      </c>
+      <c r="B13" s="27" t="s">
         <v>275</v>
       </c>
-      <c r="B6" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="33" t="s">
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+    </row>
+    <row r="14" spans="1:4" ht="27">
+      <c r="A14" s="31" t="s">
+        <v>266</v>
+      </c>
+      <c r="B14" s="27" t="s">
         <v>276</v>
       </c>
-      <c r="B7" s="29" t="s">
-        <v>292</v>
-      </c>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="33" t="s">
-        <v>277</v>
-      </c>
-      <c r="B8" s="29" t="s">
-        <v>293</v>
-      </c>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="33" t="s">
-        <v>278</v>
-      </c>
-      <c r="B9" s="29" t="s">
-        <v>294</v>
-      </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="33" t="s">
-        <v>279</v>
-      </c>
-      <c r="B10" s="29" t="s">
-        <v>294</v>
-      </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="33" t="s">
-        <v>280</v>
-      </c>
-      <c r="B11" s="29" t="s">
-        <v>294</v>
-      </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="33" t="s">
-        <v>281</v>
-      </c>
-      <c r="B12" s="29" t="s">
-        <v>295</v>
-      </c>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="33" t="s">
-        <v>286</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>296</v>
-      </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29"/>
-    </row>
-    <row r="14" spans="1:4" ht="27">
-      <c r="A14" s="33" t="s">
-        <v>287</v>
-      </c>
-      <c r="B14" s="29" t="s">
-        <v>297</v>
-      </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="29"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
     </row>
     <row r="15" spans="1:4">
-      <c r="A15" s="34" t="s">
-        <v>288</v>
-      </c>
-      <c r="B15" s="35" t="s">
-        <v>283</v>
-      </c>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
+      <c r="A15" s="32" t="s">
+        <v>267</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="36" t="s">
-        <v>282</v>
-      </c>
-      <c r="B16" s="35" t="s">
-        <v>283</v>
-      </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
+      <c r="A16" s="34" t="s">
+        <v>261</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="36" t="s">
-        <v>284</v>
-      </c>
-      <c r="B17" s="35" t="s">
-        <v>283</v>
-      </c>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
+      <c r="A17" s="34" t="s">
+        <v>263</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="36" t="s">
-        <v>285</v>
-      </c>
-      <c r="B18" s="35" t="s">
-        <v>283</v>
-      </c>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
+      <c r="A18" s="34" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>262</v>
+      </c>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>